<commit_message>
fix lỗi và test lại
</commit_message>
<xml_diff>
--- a/custom_addons/export_outgoing_picking_excel/static/template/Lenh_xuat_kho.xlsx
+++ b/custom_addons/export_outgoing_picking_excel/static/template/Lenh_xuat_kho.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atu30\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A4B9234-9752-4C28-B718-C3BC9A584C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0662DFF2-AD61-44E5-BD0F-B7986AA67D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2616" yWindow="2616" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>